<commit_message>
added second testcase. Updated some Utils methods, step definitions and page object classes.
</commit_message>
<xml_diff>
--- a/TestData/UserDetails.xlsx
+++ b/TestData/UserDetails.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anbhaduri/Desktop/My workspace/Practice_PIP/UrbanLadder/UrbanLadder/TestData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anbhaduri/Desktop/My workspace/PracticeClone/TestData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D7B55DF-3BBB-3D43-9645-7C40C77C9C83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29D5FA8E-764E-F148-9436-CC2EA0A76D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17300" xr2:uid="{5F07425E-955D-714D-BCDC-7F919BA892DE}"/>
   </bookViews>
@@ -65,7 +65,7 @@
     <t>1234567890</t>
   </si>
   <si>
-    <t>aniani@email.com</t>
+    <t>aniking@email.com</t>
   </si>
 </sst>
 </file>

</xml_diff>